<commit_message>
release: make staff study advisory
</commit_message>
<xml_diff>
--- a/tests/acceptance/staff/DCC-1.2.0-staff-acceptance.xlsx
+++ b/tests/acceptance/staff/DCC-1.2.0-staff-acceptance.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="R0bcb69deea4c4222"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参与者" sheetId="2" r:id="R6be1d07641d940dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景记录" sheetId="3" r:id="Rf14f7486e65c4cb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="区分测试" sheetId="4" r:id="Rd58cd34692d34147"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUS问卷" sheetId="5" r:id="R3368fd55bfd54e87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="签署" sheetId="6" r:id="R76b9dd64ddfc41b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分摘要" sheetId="7" r:id="R67cfa35e4e9c434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="R2c4827c4f759417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参与者" sheetId="2" r:id="R80d06c597c84462c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景记录" sheetId="3" r:id="R731d2080d23243d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="区分测试" sheetId="4" r:id="Re1f09d153e1e4bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUS问卷" sheetId="5" r:id="Rc0d4e56e8c9d48da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="签署" sheetId="6" r:id="Rd40f043aaeb4457b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分摘要" sheetId="7" r:id="R206e631dd00c4ea6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -904,7 +904,7 @@
     <x:row r="2" ht="31" customHeight="1"/>
     <x:row r="4">
       <x:c r="A4" s="8" t="str">
-        <x:v>用途：收集至少 5 名不了解统计和编程的真实调查工作人员完成严格 Excel、validation、preview、execute 和报告解释的证据。只填写黄色单元格。自动生成、主持人代签或缺少参与者确认均不能作为通过证据。</x:v>
+        <x:v>用途：收集至少 1 名不了解统计和编程的真实调查工作人员完成严格 Excel、validation、preview、execute 和报告解释的证据。只填写黄色单元格。自动生成、主持人代签或缺少参与者确认均不能作为通过证据。本研究用于改进易用性，不阻断 DCC 包发布。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1003,7 +1003,7 @@
         <x:v>由发布负责人审核评分摘要和原始记录。</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
-        <x:v>至少 5 份有效记录</x:v>
+        <x:v>至少 1 份有效记录</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="20" t="str">
-        <x:v>发布门槛</x:v>
+        <x:v>研究门槛</x:v>
       </x:c>
       <x:c r="B18" s="21" t="str">
         <x:v>要求</x:v>
@@ -1027,7 +1027,7 @@
         <x:v>有效参与者</x:v>
       </x:c>
       <x:c r="B19" s="18" t="str">
-        <x:v>至少 5</x:v>
+        <x:v>至少 1</x:v>
       </x:c>
       <x:c r="C19" s="19" t="str">
         <x:v>评分摘要</x:v>
@@ -1289,7 +1289,7 @@
     <x:row r="2" ht="31" customHeight="1"/>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
-        <x:v>时间填写为 Excel 时间值；状态、帮助次数、代码编辑和原始文件覆盖由主持人现场记录。任何代码编辑或原始文件覆盖都会阻止发布。</x:v>
+        <x:v>时间填写为 Excel 时间值；状态、帮助次数、代码编辑和原始文件覆盖由主持人现场记录。任何代码编辑或原始文件覆盖都会使工作人员研究不通过，但不会阻断 DCC 包发布。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -3764,7 +3764,7 @@
         <x:v>结果</x:v>
       </x:c>
       <x:c r="C4" s="15" t="str">
-        <x:v>发布门槛</x:v>
+        <x:v>研究门槛</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
         <x:v>状态</x:v>
@@ -3779,7 +3779,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="19" t="str">
         <x:f>IF(B5&gt;=C5,"达到","未达到")</x:f>
@@ -3791,7 +3791,7 @@
         <x:v>总体完成率</x:v>
       </x:c>
       <x:c r="B6" s="106" t="n">
-        <x:f>COUNTIF(B13:B17,7)/5</x:f>
+        <x:f>IF(B5=0,0,COUNTIFS(B13:B17,7,H13:H17,1)/B5)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="106" t="n">
@@ -3807,7 +3807,7 @@
         <x:v>区分正确率</x:v>
       </x:c>
       <x:c r="B7" s="106" t="n">
-        <x:f>SUM('区分测试'!F6:F25)/20</x:f>
+        <x:f>IF(B5=0,0,SUM(D13:D17)/B5)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="106" t="n">
@@ -3823,7 +3823,7 @@
         <x:v>SUS 中位数</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:f>MEDIAN(E13:E17)</x:f>
+        <x:f>IF(B5=0,0,MEDIAN(E13:E17))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="18" t="n">
@@ -3907,13 +3907,11 @@
         <x:f>SUMIFS('场景记录'!$F$6:$F$40,'场景记录'!$A$6:$A$40,A13)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D13" s="106" t="n">
-        <x:f>SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A13)/4</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E13" s="18" t="n">
-        <x:f>SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A13)*2.5</x:f>
-        <x:v>0</x:v>
+      <x:c r="D13" s="106" t="str">
+        <x:f>IF(H13=1,SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A13)/4,"")</x:f>
+      </x:c>
+      <x:c r="E13" s="18" t="str">
+        <x:f>IF(H13=1,SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A13)*2.5,"")</x:f>
       </x:c>
       <x:c r="F13" s="18" t="n">
         <x:f>SUMIFS('场景记录'!$I$6:$I$40,'场景记录'!$A$6:$A$40,A13)</x:f>
@@ -3944,13 +3942,11 @@
         <x:f>SUMIFS('场景记录'!$F$6:$F$40,'场景记录'!$A$6:$A$40,A14)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D14" s="106" t="n">
-        <x:f>SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A14)/4</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E14" s="18" t="n">
-        <x:f>SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A14)*2.5</x:f>
-        <x:v>0</x:v>
+      <x:c r="D14" s="106" t="str">
+        <x:f>IF(H14=1,SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A14)/4,"")</x:f>
+      </x:c>
+      <x:c r="E14" s="18" t="str">
+        <x:f>IF(H14=1,SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A14)*2.5,"")</x:f>
       </x:c>
       <x:c r="F14" s="18" t="n">
         <x:f>SUMIFS('场景记录'!$I$6:$I$40,'场景记录'!$A$6:$A$40,A14)</x:f>
@@ -3981,13 +3977,11 @@
         <x:f>SUMIFS('场景记录'!$F$6:$F$40,'场景记录'!$A$6:$A$40,A15)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D15" s="106" t="n">
-        <x:f>SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A15)/4</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E15" s="18" t="n">
-        <x:f>SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A15)*2.5</x:f>
-        <x:v>0</x:v>
+      <x:c r="D15" s="106" t="str">
+        <x:f>IF(H15=1,SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A15)/4,"")</x:f>
+      </x:c>
+      <x:c r="E15" s="18" t="str">
+        <x:f>IF(H15=1,SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A15)*2.5,"")</x:f>
       </x:c>
       <x:c r="F15" s="18" t="n">
         <x:f>SUMIFS('场景记录'!$I$6:$I$40,'场景记录'!$A$6:$A$40,A15)</x:f>
@@ -4018,13 +4012,11 @@
         <x:f>SUMIFS('场景记录'!$F$6:$F$40,'场景记录'!$A$6:$A$40,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D16" s="106" t="n">
-        <x:f>SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A16)/4</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E16" s="18" t="n">
-        <x:f>SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A16)*2.5</x:f>
-        <x:v>0</x:v>
+      <x:c r="D16" s="106" t="str">
+        <x:f>IF(H16=1,SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A16)/4,"")</x:f>
+      </x:c>
+      <x:c r="E16" s="18" t="str">
+        <x:f>IF(H16=1,SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A16)*2.5,"")</x:f>
       </x:c>
       <x:c r="F16" s="18" t="n">
         <x:f>SUMIFS('场景记录'!$I$6:$I$40,'场景记录'!$A$6:$A$40,A16)</x:f>
@@ -4055,13 +4047,11 @@
         <x:f>SUMIFS('场景记录'!$F$6:$F$40,'场景记录'!$A$6:$A$40,A17)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D17" s="107" t="n">
-        <x:f>SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A17)/4</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E17" s="24" t="n">
-        <x:f>SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A17)*2.5</x:f>
-        <x:v>0</x:v>
+      <x:c r="D17" s="107" t="str">
+        <x:f>IF(H17=1,SUMIFS('区分测试'!$F$6:$F$25,'区分测试'!$A$6:$A$25,A17)/4,"")</x:f>
+      </x:c>
+      <x:c r="E17" s="24" t="str">
+        <x:f>IF(H17=1,SUMIFS('SUS问卷'!$E$6:$E$55,'SUS问卷'!$A$6:$A$55,A17)*2.5,"")</x:f>
       </x:c>
       <x:c r="F17" s="24" t="n">
         <x:f>SUMIFS('场景记录'!$I$6:$I$40,'场景记录'!$A$6:$A$40,A17)</x:f>
@@ -4082,13 +4072,13 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="10" t="str">
-        <x:v>发布状态</x:v>
+        <x:v>工作人员流程状态</x:v>
       </x:c>
       <x:c r="B20"/>
       <x:c r="C20"/>
       <x:c r="D20"/>
       <x:c r="E20" s="109" t="str">
-        <x:f>IF(B5&lt;5,"facilitator_required",IF(AND(B6&gt;=0.8,B7&gt;=0.8,B8&gt;=75,B9=0,B10=0),"pass","fail"))</x:f>
+        <x:f>IF(B5&lt;1,"facilitator_required",IF(AND(B6&gt;=0.8,B7&gt;=0.8,B8&gt;=75,B9=0,B10=0),"pass","fail"))</x:f>
         <x:v>facilitator_required</x:v>
       </x:c>
     </x:row>
@@ -4097,7 +4087,7 @@
         <x:v>此工作簿不包含真实人员结果。参与者、主持人、签名、日期、时间、答案和评分均须在真实测试中填写；发布负责人须复核原始证据和 SHA-256。</x:v>
       </x:c>
       <x:c r="B21" t="str">
-        <x:v>只有至少 5 份有效签署记录且所有总体门槛达到时才显示 pass。当前空白模板必须保持 facilitator_required。</x:v>
+        <x:v>至少 1 份有效签署记录且所有总体门槛达到时显示 pass。当前空白模板保持 facilitator_required。此状态仅用于易用性改进，不阻断 DCC 包发布。</x:v>
       </x:c>
       <x:c r="C21"/>
       <x:c r="D21"/>

</xml_diff>